<commit_message>
Actualizar raw de Kobo - Conservando Atitlán
</commit_message>
<xml_diff>
--- a/data_raw/conservando_atitlan/kobo_mensual_raw.xlsx
+++ b/data_raw/conservando_atitlan/kobo_mensual_raw.xlsx
@@ -7,7 +7,11 @@
     <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Conservando Atitlán - Report..." sheetId="1" r:id="rId1"/>
+    <sheet name="rep_jornada" sheetId="2" r:id="rId2"/>
+    <sheet name="rep_produccion" sheetId="3" r:id="rId3"/>
+    <sheet name="rep_ventas" sheetId="4" r:id="rId4"/>
+    <sheet name="rep_actividad" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -340,9 +344,1302 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
+  <dimension ref="A1:BF2"/>
   <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>start</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>end</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>today</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>deviceid</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>username</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>programa_id</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>programa_nombre</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>intro</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>anio_reportado</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>nota_anio_fijo</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>mes_reportado</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>mes_num</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>estado_reporte</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>periodo_clave</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>observaciones_generales</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>modulos_activos</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>modulos_activos/recoleccion</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>modulos_activos/produccion</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>modulos_activos/ventas</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>modulos_activos/complementarias</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>nota_modulos</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>nota_recoleccion</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>jornadas_mes</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>aceite_litros_mes</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>agua_protegida_mes</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>inmuebles_atendidos_mes</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>resumen_recoleccion</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
+          <t>nota_produccion</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>hotel_producidos_mes</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
+          <t>tocador_producidos_mes</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
+          <t>jabones_producidos_mes</t>
+        </is>
+      </c>
+      <c r="AF1" t="inlineStr">
+        <is>
+          <t>resumen_produccion</t>
+        </is>
+      </c>
+      <c r="AG1" t="inlineStr">
+        <is>
+          <t>nota_ventas</t>
+        </is>
+      </c>
+      <c r="AH1" t="inlineStr">
+        <is>
+          <t>hotel_vendidos_mes</t>
+        </is>
+      </c>
+      <c r="AI1" t="inlineStr">
+        <is>
+          <t>tocador_vendidos_mes</t>
+        </is>
+      </c>
+      <c r="AJ1" t="inlineStr">
+        <is>
+          <t>ingresos_mes</t>
+        </is>
+      </c>
+      <c r="AK1" t="inlineStr">
+        <is>
+          <t>resumen_ventas</t>
+        </is>
+      </c>
+      <c r="AL1" t="inlineStr">
+        <is>
+          <t>nota_complementarias</t>
+        </is>
+      </c>
+      <c r="AM1" t="inlineStr">
+        <is>
+          <t>actividades_mes</t>
+        </is>
+      </c>
+      <c r="AN1" t="inlineStr">
+        <is>
+          <t>resumen_actividades</t>
+        </is>
+      </c>
+      <c r="AO1" t="inlineStr">
+        <is>
+          <t>nota_revision_1</t>
+        </is>
+      </c>
+      <c r="AP1" t="inlineStr">
+        <is>
+          <t>meta_anual_jornadas</t>
+        </is>
+      </c>
+      <c r="AQ1" t="inlineStr">
+        <is>
+          <t>meta_anual_aceite</t>
+        </is>
+      </c>
+      <c r="AR1" t="inlineStr">
+        <is>
+          <t>meta_anual_agua</t>
+        </is>
+      </c>
+      <c r="AS1" t="inlineStr">
+        <is>
+          <t>meta_anual_jabones</t>
+        </is>
+      </c>
+      <c r="AT1" t="inlineStr">
+        <is>
+          <t>nota_revision_2</t>
+        </is>
+      </c>
+      <c r="AU1" t="inlineStr">
+        <is>
+          <t>comentarios_revision</t>
+        </is>
+      </c>
+      <c r="AV1" t="inlineStr">
+        <is>
+          <t>_id</t>
+        </is>
+      </c>
+      <c r="AW1" t="inlineStr">
+        <is>
+          <t>_uuid</t>
+        </is>
+      </c>
+      <c r="AX1" t="inlineStr">
+        <is>
+          <t>_submission_time</t>
+        </is>
+      </c>
+      <c r="AY1" t="inlineStr">
+        <is>
+          <t>_validation_status</t>
+        </is>
+      </c>
+      <c r="AZ1" t="inlineStr">
+        <is>
+          <t>_notes</t>
+        </is>
+      </c>
+      <c r="BA1" t="inlineStr">
+        <is>
+          <t>_status</t>
+        </is>
+      </c>
+      <c r="BB1" t="inlineStr">
+        <is>
+          <t>_submitted_by</t>
+        </is>
+      </c>
+      <c r="BC1" t="inlineStr">
+        <is>
+          <t>__version__</t>
+        </is>
+      </c>
+      <c r="BD1" t="inlineStr">
+        <is>
+          <t>_tags</t>
+        </is>
+      </c>
+      <c r="BE1" t="inlineStr">
+        <is>
+          <t>meta/rootUuid</t>
+        </is>
+      </c>
+      <c r="BF1" t="inlineStr">
+        <is>
+          <t>_index</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-03-12T23:13:55.171-06:00</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-03-12T23:16:20.581-06:00</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2026-03-11</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>ee.kobotoolbox.org:U6VBRZrqozC5JwCT</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>username not found</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>conservando_atitlan</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Conservando Atitlán</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>mar</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>final_validado</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>2026-mar</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>recoleccion produccion ventas complementarias</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>300000</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="AC2" t="inlineStr">
+        <is>
+          <t>3000</t>
+        </is>
+      </c>
+      <c r="AD2" t="inlineStr">
+        <is>
+          <t>2345</t>
+        </is>
+      </c>
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t>5345</t>
+        </is>
+      </c>
+      <c r="AH2" t="inlineStr">
+        <is>
+          <t>400</t>
+        </is>
+      </c>
+      <c r="AI2" t="inlineStr">
+        <is>
+          <t>344</t>
+        </is>
+      </c>
+      <c r="AJ2" t="inlineStr">
+        <is>
+          <t>9160</t>
+        </is>
+      </c>
+      <c r="AM2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AP2" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="AQ2" t="inlineStr">
+        <is>
+          <t>80000</t>
+        </is>
+      </c>
+      <c r="AR2" t="inlineStr">
+        <is>
+          <t>80000000</t>
+        </is>
+      </c>
+      <c r="AS2" t="inlineStr">
+        <is>
+          <t>65040</t>
+        </is>
+      </c>
+      <c r="AV2">
+        <v>695421776</v>
+      </c>
+      <c r="AW2" t="inlineStr">
+        <is>
+          <t>85e104dd-19aa-4b8c-9872-29d9ecdc33c6</t>
+        </is>
+      </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>2026-03-13T05:16:20</t>
+        </is>
+      </c>
+      <c r="BA2" t="inlineStr">
+        <is>
+          <t>submitted_via_web</t>
+        </is>
+      </c>
+      <c r="BC2" t="inlineStr">
+        <is>
+          <t>vFdMNjMQdckWoSdfXyamyU</t>
+        </is>
+      </c>
+      <c r="BE2" t="inlineStr">
+        <is>
+          <t>uuid:85e104dd-19aa-4b8c-9872-29d9ecdc33c6</t>
+        </is>
+      </c>
+      <c r="BF2">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:V2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>fecha_jornada</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>responsable_jornada</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>municipios_visitados_texto</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>num_municipios_visitados</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>inmuebles_atendidos</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>litros_aceite_jornada</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>foto_jornada</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>observaciones_jornada</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>agua_protegida_jornada</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>_index</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>_parent_table_name</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>_parent_index</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>_submission__id</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>_submission__uuid</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>_submission__submission_time</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>_submission__validation_status</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>_submission__notes</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>_submission__status</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>_submission__submitted_by</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>_submission___version__</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>_submission__tags</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>_submission_meta/rootUuid</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-03-03</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Julio Romero</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>San Juan La Laguna</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>300000</t>
+        </is>
+      </c>
+      <c r="J2">
+        <v>1</v>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Conservando Atitlán - Reporte mensual único</t>
+        </is>
+      </c>
+      <c r="L2">
+        <v>1</v>
+      </c>
+      <c r="M2">
+        <v>695421776</v>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>85e104dd-19aa-4b8c-9872-29d9ecdc33c6</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>2026-03-13T05:16:20</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>submitted_via_web</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>vFdMNjMQdckWoSdfXyamyU</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>uuid:85e104dd-19aa-4b8c-9872-29d9ecdc33c6</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:V2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>fecha_produccion</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>responsable_produccion</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>codigo_lote</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>litros_aceite_utilizados</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>hotel_producidos</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>tocador_producidos</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>foto_produccion</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>observaciones_produccion</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>jabones_oficiales_lote</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>_index</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>_parent_table_name</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>_parent_index</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>_submission__id</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>_submission__uuid</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>_submission__submission_time</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>_submission__validation_status</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>_submission__notes</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>_submission__status</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>_submission__submitted_by</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>_submission___version__</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>_submission__tags</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>_submission_meta/rootUuid</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-03-13</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Sharon</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>3435</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>245</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>3000</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>2345</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>5345</t>
+        </is>
+      </c>
+      <c r="J2">
+        <v>1</v>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Conservando Atitlán - Reporte mensual único</t>
+        </is>
+      </c>
+      <c r="L2">
+        <v>1</v>
+      </c>
+      <c r="M2">
+        <v>695421776</v>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>85e104dd-19aa-4b8c-9872-29d9ecdc33c6</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>2026-03-13T05:16:20</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>submitted_via_web</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>vFdMNjMQdckWoSdfXyamyU</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>uuid:85e104dd-19aa-4b8c-9872-29d9ecdc33c6</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:AA2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>fecha_venta</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>tipo_cliente</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>cliente_nombre</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>factura_referencia</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>fuente_precio</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>hotel_vendidos</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>precio_hotel_unit</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>subtotal_hotel</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>tocador_vendidos</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>precio_tocador_unit</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>subtotal_tocador</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>total_venta</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>comprobante_venta</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>observaciones_venta</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>_index</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>_parent_table_name</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>_parent_index</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>_submission__id</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>_submission__uuid</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>_submission__submission_time</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>_submission__validation_status</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>_submission__notes</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>_submission__status</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>_submission__submitted_by</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>_submission___version__</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>_submission__tags</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>_submission_meta/rootUuid</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>hotel</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Porta Hotel del Lago</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>tabla_descuentos</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>400</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>4000</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>344</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>5160</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>9160</t>
+        </is>
+      </c>
+      <c r="O2">
+        <v>1</v>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Conservando Atitlán - Reporte mensual único</t>
+        </is>
+      </c>
+      <c r="Q2">
+        <v>1</v>
+      </c>
+      <c r="R2">
+        <v>695421776</v>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>85e104dd-19aa-4b8c-9872-29d9ecdc33c6</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>2026-03-13T05:16:20</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>submitted_via_web</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>vFdMNjMQdckWoSdfXyamyU</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>uuid:85e104dd-19aa-4b8c-9872-29d9ecdc33c6</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:S2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>fecha_actividad</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>tipo_actividad</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>cantidad_actividad</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>municipio_actividad</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>descripcion_actividad</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>evidencia_actividad</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>_index</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>_parent_table_name</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>_parent_index</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>_submission__id</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>_submission__uuid</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>_submission__submission_time</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>_submission__validation_status</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>_submission__notes</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>_submission__status</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>_submission__submitted_by</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>_submission___version__</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>_submission__tags</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>_submission_meta/rootUuid</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>publicacion_redes</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>San Juan La Laguna</t>
+        </is>
+      </c>
+      <c r="G2">
+        <v>1</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Conservando Atitlán - Reporte mensual único</t>
+        </is>
+      </c>
+      <c r="I2">
+        <v>1</v>
+      </c>
+      <c r="J2">
+        <v>695421776</v>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>85e104dd-19aa-4b8c-9872-29d9ecdc33c6</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>2026-03-13T05:16:20</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>submitted_via_web</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>vFdMNjMQdckWoSdfXyamyU</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>uuid:85e104dd-19aa-4b8c-9872-29d9ecdc33c6</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>